<commit_message>
260905 0512 modification push
</commit_message>
<xml_diff>
--- a/evaluation/rq2/rq2a_specification_profile.xlsx
+++ b/evaluation/rq2/rq2a_specification_profile.xlsx
@@ -3801,7 +3801,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>gamma</t>
+          <t>alpha_and_beta</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -3852,7 +3852,7 @@
       </c>
       <c r="AH29" t="inlineStr">
         <is>
-          <t>Doc gives a clear vocabulary mapping: an initial reclassification attempt to L5b used a '@During uToken.transferFrom.arg[2] == premiumFilled' proxy annotation (grammar-expressible, distinguishes buggy/correct formally), but this was withdrawn on the grounds that the true intent (sender's net token flow = an external ERC20 balanceOf entry-exit difference, outside Swivel's own scope) cannot itself be expressed, and the arg[2] relation is only a proxy that happens to work, not a direct statement of intent. Doc's root-cause section explicitly assigns this case a new axis label 'axis γ — multi-point accounting cannot be captured by a single-point annotation' (the bug spans two separate transferFrom calls whose combined net effect, not either call alone, is what's wrong), matching csv's l4a_axis=gamma directly. Also flags a natspec-driven silent-sanction risk: the in-code comment above the buggy line states the buggy behavior verbatim, so a developer following it would write the wrong intent as-is.</t>
+          <t>Doc gives a clear vocabulary mapping: an initial reclassification attempt to L5b used a '@During uToken.transferFrom.arg[2] == premiumFilled' proxy annotation (grammar-expressible, distinguishes buggy/correct formally), but this was withdrawn on the grounds that the true intent (sender's net token flow = an external ERC20 balanceOf entry-exit difference, outside Swivel's own scope) cannot itself be expressed, and the arg[2] relation is only a proxy that happens to work, not a direct statement of intent. Doc's root-cause section explicitly assigns this case a new axis label 'axis γ — multi-point accounting cannot be captured by a single-point annotation' (the bug spans two separate transferFrom calls whose combined net effect, not either call alone, is what's wrong), matching csv's l4a_axis=gamma directly. Also flags a natspec-driven silent-sanction risk: the in-code comment above the buggy line states the buggy behavior verbatim, so a developer following it would write the wrong intent as-is. | RETAG (2026-09-05): blocker_tags corrected gamma-&gt;alpha_and_beta. Source doc (l4_l5_case_review Case 4) concluded L4a with G1 (external balanceOf call needed, alpha) + G3 (no in-scope var holds net flow, beta); the doc's own 'axis γ' label was an old internal L4a sub-axis ('multi-point accounting'), not the new methodology's gamma (relation-form/grammar-arithmetic). Mechanical mapping of that string to the new gamma tag was a mislabel.</t>
         </is>
       </c>
     </row>
@@ -5851,7 +5851,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>gamma</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="H47" t="inlineStr"/>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="AH47" t="inlineStr">
         <is>
-          <t>csv l4a_axis blank (L4b, not L4a); primary_G=G1;G3;G4. Case review frames the primary blocker as a call-ordering defect -- _push() must call updateTvls() BEFORE the deposit accounting, not after -- and states explicitly this 'ordering 문제가 단일 annotation 범위 넘음' (the ordering problem exceeds a single annotation's scope). Mapped this to gamma (relation is inherently multi-point/structural, spans the relative order of two statements/calls, not capturable by any single-relation form) since that's the closest fit in the R1-7 vocabulary, though the doc does not itself use alpha/beta/gamma/delta terms (this case review predates that vocabulary). csv also carries G1 in primary_G, suggesting a possible secondary alpha component (a function-call result involved), but the case-review prose centers entirely on the ordering/sequencing problem, not on any single unreferenceable call result -- flagging low-to-moderate confidence on whether a secondary alpha tag should also apply.</t>
+          <t>csv l4a_axis blank (L4b, not L4a); primary_G=G1;G3;G4. Case review frames the primary blocker as a call-ordering defect -- _push() must call updateTvls() BEFORE the deposit accounting, not after -- and states explicitly this 'ordering 문제가 단일 annotation 범위 넘음' (the ordering problem exceeds a single annotation's scope). Mapped this to gamma (relation is inherently multi-point/structural, spans the relative order of two statements/calls, not capturable by any single-relation form) since that's the closest fit in the R1-7 vocabulary, though the doc does not itself use alpha/beta/gamma/delta terms (this case review predates that vocabulary). csv also carries G1 in primary_G, suggesting a possible secondary alpha component (a function-call result involved), but the case-review prose centers entirely on the ordering/sequencing problem, not on any single unreferenceable call result -- flagging low-to-moderate confidence on whether a secondary alpha tag should also apply. | RETAG (2026-09-05): blocker_tags corrected gamma-&gt;beta. Source doc (l4_l5_case_review Case 16) is proxy_type=B, L4b family (Type-B-only cell): no in-scope value tracks whether updateTvls() ran before the deposit (ordering fact absent from scope entirely, not a grammar-arithmetic limitation); consistent with sibling L4b cases already tagged beta. Already-Unusable status is unchanged and now consistent with the alpha/beta-implies-Unusable pattern.</t>
         </is>
       </c>
     </row>
@@ -20244,7 +20244,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="80">
@@ -20264,7 +20264,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="82">
@@ -20294,7 +20294,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>